<commit_message>
Assessment criteria, version 1.1: instructions, MQA indicators, sources and thresholds
</commit_message>
<xml_diff>
--- a/criteria/criteria.xlsx
+++ b/criteria/criteria.xlsx
@@ -11,7 +11,7 @@
     <sheet name="About" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Criteria'!$A$1:$O$24</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Criteria'!$A$1:$R$24</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'Criteria'!$1:$1</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -464,24 +464,27 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:O24"/>
+  <dimension ref="A1:R24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
     <col width="22" customWidth="1" min="3" max="3"/>
     <col width="7" customWidth="1" min="4" max="4"/>
-    <col width="34" customWidth="1" min="5" max="5"/>
-    <col width="40" customWidth="1" min="6" max="6"/>
+    <col width="30" customWidth="1" min="5" max="5"/>
+    <col width="34" customWidth="1" min="6" max="6"/>
     <col width="40" customWidth="1" min="7" max="7"/>
     <col width="40" customWidth="1" min="8" max="8"/>
-    <col width="28" customWidth="1" min="9" max="9"/>
-    <col width="16" customWidth="1" min="10" max="10"/>
-    <col width="48" customWidth="1" min="11" max="11"/>
-    <col width="11" customWidth="1" min="12" max="12"/>
-    <col width="28" customWidth="1" min="13" max="13"/>
-    <col width="36" customWidth="1" min="14" max="14"/>
-    <col width="7" customWidth="1" min="15" max="15"/>
+    <col width="40" customWidth="1" min="9" max="9"/>
+    <col width="28" customWidth="1" min="10" max="10"/>
+    <col width="16" customWidth="1" min="11" max="11"/>
+    <col width="48" customWidth="1" min="12" max="12"/>
+    <col width="11" customWidth="1" min="13" max="13"/>
+    <col width="28" customWidth="1" min="14" max="14"/>
+    <col width="36" customWidth="1" min="15" max="15"/>
+    <col width="7" customWidth="1" min="16" max="16"/>
+    <col width="34" customWidth="1" min="17" max="17"/>
+    <col width="34" customWidth="1" min="18" max="18"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -507,57 +510,72 @@
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
+          <t>Instruction</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
           <t>Question</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Score 0</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Score 1</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Score 2</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Not applicable</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>Method</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>How to check</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>Applies to</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>Typical fix</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>Sources</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>FAIR</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>MQA (data.gov.gr)</t>
+        </is>
+      </c>
+      <c r="R1" s="1" t="inlineStr">
+        <is>
+          <t>MQA (data.europa.eu)</t>
         </is>
       </c>
     </row>
@@ -584,53 +602,68 @@
       </c>
       <c r="E2" s="3" t="inlineStr">
         <is>
+          <t>Addition: ISO/IEC 25012 (availability)</t>
+        </is>
+      </c>
+      <c r="F2" s="3" t="inlineStr">
+        <is>
           <t>Can the dataset's own resources be downloaded and opened?</t>
         </is>
       </c>
-      <c r="F2" s="3" t="inlineStr">
+      <c r="G2" s="3" t="inlineStr">
         <is>
           <t>No resource can be downloaded or opened.</t>
         </is>
       </c>
-      <c r="G2" s="3" t="inlineStr">
+      <c r="H2" s="3" t="inlineStr">
         <is>
           <t>At least one resource can be downloaded and opened, but at least one other fails (broken link, error page, empty or wrong file).</t>
         </is>
       </c>
-      <c r="H2" s="3" t="inlineStr">
+      <c r="I2" s="3" t="inlineStr">
         <is>
           <t>Every resource can be downloaded and opens without error.</t>
         </is>
       </c>
-      <c r="I2" s="3" t="inlineStr"/>
-      <c r="J2" s="3" t="inlineStr">
+      <c r="J2" s="3" t="inlineStr"/>
+      <c r="K2" s="3" t="inlineStr">
         <is>
           <t>automatic, confirmed manually</t>
         </is>
       </c>
-      <c r="K2" s="3" t="inlineStr">
+      <c r="L2" s="3" t="inlineStr">
         <is>
           <t>Download test of every resource except the portal's 'download all' bundle, repeated on a second day before a failure is recorded (fact sheet). A link that leads to a web page instead of the declared file counts as a failure.</t>
         </is>
       </c>
-      <c r="L2" s="3" t="inlineStr">
+      <c r="M2" s="3" t="inlineStr">
         <is>
           <t>all</t>
         </is>
       </c>
-      <c r="M2" s="3" t="inlineStr">
+      <c r="N2" s="3" t="inlineStr">
         <is>
           <t>Low: correct the link. Medium: restore or upload the file again.</t>
         </is>
       </c>
-      <c r="N2" s="3" t="inlineStr">
+      <c r="O2" s="3" t="inlineStr">
         <is>
           <t>ISO/IEC 25012:2008 (availability)</t>
         </is>
       </c>
-      <c r="O2" s="3" t="inlineStr">
+      <c r="P2" s="3" t="inlineStr">
         <is>
           <t>A1</t>
+        </is>
+      </c>
+      <c r="Q2" s="3" t="inlineStr">
+        <is>
+          <t>Accessibility: access URL accessibility; download URL accessibility</t>
+        </is>
+      </c>
+      <c r="R2" s="3" t="inlineStr">
+        <is>
+          <t>Distribution: access URL accessibility test; download URL accessibility test</t>
         </is>
       </c>
     </row>
@@ -657,61 +690,76 @@
       </c>
       <c r="E3" s="4" t="inlineStr">
         <is>
+          <t>Level (a): completeness</t>
+        </is>
+      </c>
+      <c r="F3" s="4" t="inlineStr">
+        <is>
           <t>How many values are missing?</t>
         </is>
       </c>
-      <c r="F3" s="4" t="inlineStr">
+      <c r="G3" s="4" t="inlineStr">
         <is>
           <t>More than 20% of the cells are empty, or no file can be opened.</t>
         </is>
       </c>
-      <c r="G3" s="4" t="inlineStr">
+      <c r="H3" s="4" t="inlineStr">
         <is>
           <t>5-20% of the cells are empty, or at least one column is entirely empty.</t>
         </is>
       </c>
-      <c r="H3" s="4" t="inlineStr">
+      <c r="I3" s="4" t="inlineStr">
         <is>
           <t>Less than 5% of the cells are empty and no column is entirely empty.</t>
         </is>
       </c>
-      <c r="I3" s="4" t="inlineStr">
+      <c r="J3" s="4" t="inlineStr">
         <is>
           <t>The resources contain no records or attributes, e.g. a raster image or a scanned map; the reason is recorded.</t>
         </is>
       </c>
-      <c r="J3" s="4" t="inlineStr">
+      <c r="K3" s="4" t="inlineStr">
         <is>
           <t>automatic for machine-readable files; manual otherwise</t>
         </is>
       </c>
-      <c r="K3" s="4" t="inlineStr">
+      <c r="L3" s="4" t="inlineStr">
         <is>
           <t>Share of empty cells in the most recent machine-readable file (fact sheet). Placeholders such as '-', 'N/A' or '..' count as empty. For data published only as documents (e.g. tables in PDF), estimated by inspection.</t>
         </is>
       </c>
-      <c r="L3" s="4" t="inlineStr">
+      <c r="M3" s="4" t="inlineStr">
         <is>
           <t>all</t>
         </is>
       </c>
-      <c r="M3" s="4" t="inlineStr">
+      <c r="N3" s="4" t="inlineStr">
         <is>
           <t>Medium: complete the file or state why values are missing.</t>
         </is>
       </c>
-      <c r="N3" s="4" t="inlineStr">
-        <is>
-          <t>ISO/IEC 25012:2008 (completeness)</t>
-        </is>
-      </c>
       <c r="O3" s="4" t="inlineStr">
         <is>
+          <t>ISO/IEC 25012:2008 (completeness); Publications Office of the EU (2021), data.europa.eu data quality guidelines, section 1.1.1.2</t>
+        </is>
+      </c>
+      <c r="P3" s="4" t="inlineStr">
+        <is>
           <t>R1</t>
         </is>
       </c>
-    </row>
-    <row r="4" ht="64" customHeight="1">
+      <c r="Q3" s="4" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="R3" s="4" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="94" customHeight="1">
       <c r="A4" s="4" t="inlineStr">
         <is>
           <t>Q3</t>
@@ -734,57 +782,72 @@
       </c>
       <c r="E4" s="4" t="inlineStr">
         <is>
+          <t>Level (a): consistency</t>
+        </is>
+      </c>
+      <c r="F4" s="4" t="inlineStr">
+        <is>
           <t>Are the values recorded in the same way throughout the dataset?</t>
         </is>
       </c>
-      <c r="F4" s="4" t="inlineStr">
+      <c r="G4" s="4" t="inlineStr">
         <is>
           <t>Inconsistencies that prevent analysis without manual work (e.g. values shifted between columns, different units mixed in one column), or no file can be opened.</t>
         </is>
       </c>
-      <c r="G4" s="4" t="inlineStr">
+      <c r="H4" s="4" t="inlineStr">
         <is>
           <t>Minor inconsistencies: mixed date or number formats in a column, numbers stored as text, different column names or order between files of the same dataset.</t>
         </is>
       </c>
-      <c r="H4" s="4" t="inlineStr">
+      <c r="I4" s="4" t="inlineStr">
         <is>
           <t>Each column has one type, format and unit, and all files of the dataset share the same structure.</t>
         </is>
       </c>
-      <c r="I4" s="4" t="inlineStr">
+      <c r="J4" s="4" t="inlineStr">
         <is>
           <t>The resources contain no records or attributes, e.g. a raster image or a scanned map; the reason is recorded.</t>
         </is>
       </c>
-      <c r="J4" s="4" t="inlineStr">
+      <c r="K4" s="4" t="inlineStr">
         <is>
           <t>semi-automatic</t>
         </is>
       </c>
-      <c r="K4" s="4" t="inlineStr">
+      <c r="L4" s="4" t="inlineStr">
         <is>
           <t>Column types and formats (fact sheet); comparison of the headers of the files of the dataset; inspection of a sample of rows.</t>
         </is>
       </c>
-      <c r="L4" s="4" t="inlineStr">
+      <c r="M4" s="4" t="inlineStr">
         <is>
           <t>all</t>
         </is>
       </c>
-      <c r="M4" s="4" t="inlineStr">
+      <c r="N4" s="4" t="inlineStr">
         <is>
           <t>Medium: harmonise the files.</t>
         </is>
       </c>
-      <c r="N4" s="4" t="inlineStr">
-        <is>
-          <t>ISO/IEC 25012:2008 (consistency); W3C Data on the Web Best Practices (2017), BP13</t>
-        </is>
-      </c>
       <c r="O4" s="4" t="inlineStr">
         <is>
+          <t>ISO/IEC 25012:2008 (consistency); W3C Data on the Web Best Practices (2017), BP13; Publications Office of the EU (2021), data.europa.eu data quality guidelines, sections 1.1.3.1, 1.2.1.5 and 1.2.1.6</t>
+        </is>
+      </c>
+      <c r="P4" s="4" t="inlineStr">
+        <is>
           <t>R1.3</t>
+        </is>
+      </c>
+      <c r="Q4" s="4" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="R4" s="4" t="inlineStr">
+        <is>
+          <t>None</t>
         </is>
       </c>
     </row>
@@ -811,57 +874,72 @@
       </c>
       <c r="E5" s="4" t="inlineStr">
         <is>
+          <t>Addition: ISO/IEC 25012 (accuracy)</t>
+        </is>
+      </c>
+      <c r="F5" s="4" t="inlineStr">
+        <is>
           <t>Are the values plausible?</t>
         </is>
       </c>
-      <c r="F5" s="4" t="inlineStr">
+      <c r="G5" s="4" t="inlineStr">
         <is>
           <t>Systematic errors: coordinates outside Greece or in an undeclared reference system, dates in the future, values in the wrong columns; or no file can be opened.</t>
         </is>
       </c>
-      <c r="G5" s="4" t="inlineStr">
+      <c r="H5" s="4" t="inlineStr">
         <is>
           <t>Isolated implausible values (fewer than 1% of the records), e.g. negative counts or outliers that look like typing errors.</t>
         </is>
       </c>
-      <c r="H5" s="4" t="inlineStr">
+      <c r="I5" s="4" t="inlineStr">
         <is>
           <t>No implausible values in the automatic checks and in a manual review of 10 random records.</t>
         </is>
       </c>
-      <c r="I5" s="4" t="inlineStr">
+      <c r="J5" s="4" t="inlineStr">
         <is>
           <t>The resources contain no records or attributes, e.g. a raster image or a scanned map; the reason is recorded.</t>
         </is>
       </c>
-      <c r="J5" s="4" t="inlineStr">
+      <c r="K5" s="4" t="inlineStr">
         <is>
           <t>semi-automatic</t>
         </is>
       </c>
-      <c r="K5" s="4" t="inlineStr">
+      <c r="L5" s="4" t="inlineStr">
         <is>
           <t>Range checks (fact sheet): coordinates, dates, negative values, duplicates; review of 10 random records; comparison with the publisher's website where the same figures appear. Accuracy against reality cannot be verified in general, so the criterion records plausibility.</t>
         </is>
       </c>
-      <c r="L5" s="4" t="inlineStr">
+      <c r="M5" s="4" t="inlineStr">
         <is>
           <t>all</t>
         </is>
       </c>
-      <c r="M5" s="4" t="inlineStr">
+      <c r="N5" s="4" t="inlineStr">
         <is>
           <t>Medium: correct the values. High: correct the source system.</t>
         </is>
       </c>
-      <c r="N5" s="4" t="inlineStr">
+      <c r="O5" s="4" t="inlineStr">
         <is>
           <t>ISO/IEC 25012:2008 (accuracy)</t>
         </is>
       </c>
-      <c r="O5" s="4" t="inlineStr">
+      <c r="P5" s="4" t="inlineStr">
         <is>
           <t>R1</t>
+        </is>
+      </c>
+      <c r="Q5" s="4" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="R5" s="4" t="inlineStr">
+        <is>
+          <t>None</t>
         </is>
       </c>
     </row>
@@ -888,53 +966,68 @@
       </c>
       <c r="E6" s="4" t="inlineStr">
         <is>
+          <t>Level (a): timeliness</t>
+        </is>
+      </c>
+      <c r="F6" s="4" t="inlineStr">
+        <is>
           <t>Is the dataset updated as often as its metadata declare?</t>
         </is>
       </c>
-      <c r="F6" s="4" t="inlineStr">
+      <c r="G6" s="4" t="inlineStr">
         <is>
           <t>The newest data are older than three update periods, or no frequency is declared and there has been no update for more than 12 months.</t>
         </is>
       </c>
-      <c r="G6" s="4" t="inlineStr">
+      <c r="H6" s="4" t="inlineStr">
         <is>
           <t>The newest data are one to three periods late, or no frequency is declared but the dataset was updated in the last 12 months.</t>
         </is>
       </c>
-      <c r="H6" s="4" t="inlineStr">
+      <c r="I6" s="4" t="inlineStr">
         <is>
           <t>Updated within the declared frequency (with one period of tolerance), or declared as not updated (one-off or historical data) with a description that says so.</t>
         </is>
       </c>
-      <c r="I6" s="4" t="inlineStr"/>
-      <c r="J6" s="4" t="inlineStr">
+      <c r="J6" s="4" t="inlineStr"/>
+      <c r="K6" s="4" t="inlineStr">
         <is>
           <t>semi-automatic</t>
         </is>
       </c>
-      <c r="K6" s="4" t="inlineStr">
+      <c r="L6" s="4" t="inlineStr">
         <is>
           <t>Declared update frequency (metadata) against the date of the newest data: the latest date inside the data where there is one, otherwise the modification date of the newest resource.</t>
         </is>
       </c>
-      <c r="L6" s="4" t="inlineStr">
+      <c r="M6" s="4" t="inlineStr">
         <is>
           <t>all</t>
         </is>
       </c>
-      <c r="M6" s="4" t="inlineStr">
+      <c r="N6" s="4" t="inlineStr">
         <is>
           <t>Low: declare the actual frequency. High: set up regular updates.</t>
         </is>
       </c>
-      <c r="N6" s="4" t="inlineStr">
+      <c r="O6" s="4" t="inlineStr">
         <is>
           <t>ISO/IEC 25012:2008 (currentness); W3C Data on the Web Best Practices (2017), BP21; DCAT-AP 3.0.1 (frequency)</t>
         </is>
       </c>
-      <c r="O6" s="4" t="inlineStr">
+      <c r="P6" s="4" t="inlineStr">
         <is>
           <t>R1</t>
+        </is>
+      </c>
+      <c r="Q6" s="4" t="inlineStr">
+        <is>
+          <t>Contextuality: date of issue; modification date (presence only)</t>
+        </is>
+      </c>
+      <c r="R6" s="4" t="inlineStr">
+        <is>
+          <t>Dataset and distribution: modification date; date of issue (presence only)</t>
         </is>
       </c>
     </row>
@@ -961,53 +1054,68 @@
       </c>
       <c r="E7" s="3" t="inlineStr">
         <is>
+          <t>Level (a): format; 5-star scale</t>
+        </is>
+      </c>
+      <c r="F7" s="3" t="inlineStr">
+        <is>
           <t>What is the most open format in which the data are offered?</t>
         </is>
       </c>
-      <c r="F7" s="3" t="inlineStr">
+      <c r="G7" s="3" t="inlineStr">
         <is>
           <t>Only unstructured formats (PDF, word-processor documents, images, web pages) or map views without data (WMS): 1 star.</t>
         </is>
       </c>
-      <c r="G7" s="3" t="inlineStr">
+      <c r="H7" s="3" t="inlineStr">
         <is>
           <t>Structured but vendor-specific formats (XLS, XLSX, SHP, MDB) or vendor-specific services (Esri REST): 2 stars.</t>
         </is>
       </c>
-      <c r="H7" s="3" t="inlineStr">
+      <c r="I7" s="3" t="inlineStr">
         <is>
           <t>At least one open, non-proprietary structured format (CSV, JSON, GeoJSON, XML, GML, KML, GeoPackage, GeoTIFF, NetCDF, RDF) or a download service in such a format (WFS, API): 3 stars or more.</t>
         </is>
       </c>
-      <c r="I7" s="3" t="inlineStr"/>
-      <c r="J7" s="3" t="inlineStr">
+      <c r="J7" s="3" t="inlineStr"/>
+      <c r="K7" s="3" t="inlineStr">
         <is>
           <t>automatic, confirmed manually</t>
         </is>
       </c>
-      <c r="K7" s="3" t="inlineStr">
+      <c r="L7" s="3" t="inlineStr">
         <is>
           <t>Formats of the resources (fact sheet), checked against the actual content of the files: a file declared as CSV that is in fact a PDF counts as PDF.</t>
         </is>
       </c>
-      <c r="L7" s="3" t="inlineStr">
+      <c r="M7" s="3" t="inlineStr">
         <is>
           <t>all</t>
         </is>
       </c>
-      <c r="M7" s="3" t="inlineStr">
+      <c r="N7" s="3" t="inlineStr">
         <is>
           <t>Medium: publish an open format next to the existing one.</t>
         </is>
       </c>
-      <c r="N7" s="3" t="inlineStr">
-        <is>
-          <t>5-star Open Data (Berners-Lee); W3C Data on the Web Best Practices (2017), BP12 and BP14; Directive (EU) 2019/1024, Art. 5</t>
-        </is>
-      </c>
       <c r="O7" s="3" t="inlineStr">
         <is>
+          <t>5-star Open Data (Berners-Lee); W3C Data on the Web Best Practices (2017), BP12 and BP14; Directive (EU) 2019/1024, Art. 5; Circular 24849/2026, section 1.5</t>
+        </is>
+      </c>
+      <c r="P7" s="3" t="inlineStr">
+        <is>
           <t>I1</t>
+        </is>
+      </c>
+      <c r="Q7" s="3" t="inlineStr">
+        <is>
+          <t>Interoperability: format; machine readable; non-proprietary</t>
+        </is>
+      </c>
+      <c r="R7" s="3" t="inlineStr">
+        <is>
+          <t>Distribution: non-proprietary; machine readable</t>
         </is>
       </c>
     </row>
@@ -1034,57 +1142,72 @@
       </c>
       <c r="E8" s="6" t="inlineStr">
         <is>
+          <t>Level (b): DCAT-AP (mandatory properties)</t>
+        </is>
+      </c>
+      <c r="F8" s="6" t="inlineStr">
+        <is>
           <t>Are the metadata that DCAT-AP makes mandatory present and meaningful?</t>
         </is>
       </c>
-      <c r="F8" s="6" t="inlineStr">
+      <c r="G8" s="6" t="inlineStr">
         <is>
           <t>A mandatory element is missing: title, description, or an access URL for a resource.</t>
         </is>
       </c>
-      <c r="G8" s="6" t="inlineStr">
+      <c r="H8" s="6" t="inlineStr">
         <is>
           <t>All are present, but the description repeats the title or is shorter than 100 characters.</t>
         </is>
       </c>
-      <c r="H8" s="6" t="inlineStr">
+      <c r="I8" s="6" t="inlineStr">
         <is>
           <t>Title, a meaningful description (at least 100 characters, saying what the data contain) and an access URL for every resource.</t>
         </is>
       </c>
-      <c r="I8" s="6" t="inlineStr"/>
-      <c r="J8" s="6" t="inlineStr">
+      <c r="J8" s="6" t="inlineStr"/>
+      <c r="K8" s="6" t="inlineStr">
         <is>
           <t>automatic, confirmed manually</t>
         </is>
       </c>
-      <c r="K8" s="6" t="inlineStr">
+      <c r="L8" s="6" t="inlineStr">
         <is>
           <t>Portal metadata (fact sheet): title, length of the description, access URL of each resource. Whether the description is meaningful is confirmed by reading it.</t>
         </is>
       </c>
-      <c r="L8" s="6" t="inlineStr">
+      <c r="M8" s="6" t="inlineStr">
         <is>
           <t>all</t>
         </is>
       </c>
-      <c r="M8" s="6" t="inlineStr">
+      <c r="N8" s="6" t="inlineStr">
         <is>
           <t>Low: complete the metadata.</t>
         </is>
       </c>
-      <c r="N8" s="6" t="inlineStr">
+      <c r="O8" s="6" t="inlineStr">
         <is>
           <t>DCAT-AP 3.0.1 (mandatory properties of Dataset and Distribution); Ministerial Decision 11654/2026</t>
         </is>
       </c>
-      <c r="O8" s="6" t="inlineStr">
+      <c r="P8" s="6" t="inlineStr">
         <is>
           <t>F2</t>
         </is>
       </c>
-    </row>
-    <row r="9" ht="79" customHeight="1">
+      <c r="Q8" s="6" t="inlineStr">
+        <is>
+          <t>Interoperability: DCAT-AP compliance</t>
+        </is>
+      </c>
+      <c r="R8" s="6" t="inlineStr">
+        <is>
+          <t>Dataset: title; description. Distribution: access URL</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="169" customHeight="1">
       <c r="A9" s="4" t="inlineStr">
         <is>
           <t>M2</t>
@@ -1107,53 +1230,68 @@
       </c>
       <c r="E9" s="4" t="inlineStr">
         <is>
+          <t>Level (b): DCAT-AP (recommended properties)</t>
+        </is>
+      </c>
+      <c r="F9" s="4" t="inlineStr">
+        <is>
           <t>How many of seven descriptive metadata are present: keyword, theme, publisher, contact point, geographical coverage, temporal coverage, update frequency?</t>
         </is>
       </c>
-      <c r="F9" s="4" t="inlineStr">
+      <c r="G9" s="4" t="inlineStr">
         <is>
           <t>Two or fewer.</t>
         </is>
       </c>
-      <c r="G9" s="4" t="inlineStr">
+      <c r="H9" s="4" t="inlineStr">
         <is>
           <t>Three to five.</t>
         </is>
       </c>
-      <c r="H9" s="4" t="inlineStr">
+      <c r="I9" s="4" t="inlineStr">
         <is>
           <t>Six or seven.</t>
         </is>
       </c>
-      <c r="I9" s="4" t="inlineStr"/>
-      <c r="J9" s="4" t="inlineStr">
+      <c r="J9" s="4" t="inlineStr"/>
+      <c r="K9" s="4" t="inlineStr">
         <is>
           <t>automatic</t>
         </is>
       </c>
-      <c r="K9" s="4" t="inlineStr">
-        <is>
-          <t>Portal metadata (fact sheet). The first six are recommended properties of DCAT-AP; the update frequency is optional in DCAT-AP and is checked because the assessment of timeliness (Q5) depends on it.</t>
-        </is>
-      </c>
       <c r="L9" s="4" t="inlineStr">
         <is>
+          <t>Portal metadata (fact sheet). The first six are recommended properties of DCAT-AP; the update frequency is optional in DCAT-AP and is checked because the assessment of timeliness (Q5) depends on it. Geographical coverage is the area to which the data refer; for national data, the country (Greece) is sufficient. A property counts as present whenever it holds a value, including a broad, default or erroneous one (e.g. the whole of Greece for local data, a temporal coverage from 1900 to 2099, a bounding box of the whole world or outside Greece).</t>
+        </is>
+      </c>
+      <c r="M9" s="4" t="inlineStr">
+        <is>
           <t>all</t>
         </is>
       </c>
-      <c r="M9" s="4" t="inlineStr">
+      <c r="N9" s="4" t="inlineStr">
         <is>
           <t>Low: complete the metadata.</t>
         </is>
       </c>
-      <c r="N9" s="4" t="inlineStr">
+      <c r="O9" s="4" t="inlineStr">
         <is>
           <t>DCAT-AP 3.0.1; W3C Data on the Web Best Practices (2017), BP1 and BP2; Circular 24849/2026</t>
         </is>
       </c>
-      <c r="O9" s="4" t="inlineStr">
+      <c r="P9" s="4" t="inlineStr">
         <is>
           <t>F2</t>
+        </is>
+      </c>
+      <c r="Q9" s="4" t="inlineStr">
+        <is>
+          <t>Findability: keyword usage; categories; geo search; time-based search. Reusability: contact point; publisher</t>
+        </is>
+      </c>
+      <c r="R9" s="4" t="inlineStr">
+        <is>
+          <t>Dataset: keyword usage; categories; geo search; temporal coverage; publisher; contact point</t>
         </is>
       </c>
     </row>
@@ -1180,53 +1318,68 @@
       </c>
       <c r="E10" s="4" t="inlineStr">
         <is>
+          <t>Level (b): DCAT-AP (controlled vocabularies)</t>
+        </is>
+      </c>
+      <c r="F10" s="4" t="inlineStr">
+        <is>
           <t>Are theme, file format and update frequency given with terms of the controlled vocabularies?</t>
         </is>
       </c>
-      <c r="F10" s="4" t="inlineStr">
+      <c r="G10" s="4" t="inlineStr">
         <is>
           <t>None of them.</t>
         </is>
       </c>
-      <c r="G10" s="4" t="inlineStr">
+      <c r="H10" s="4" t="inlineStr">
         <is>
           <t>Some of them; the rest are free text.</t>
         </is>
       </c>
-      <c r="H10" s="4" t="inlineStr">
+      <c r="I10" s="4" t="inlineStr">
         <is>
           <t>All of those present use controlled vocabularies.</t>
         </is>
       </c>
-      <c r="I10" s="4" t="inlineStr"/>
-      <c r="J10" s="4" t="inlineStr">
+      <c r="J10" s="4" t="inlineStr"/>
+      <c r="K10" s="4" t="inlineStr">
         <is>
           <t>automatic</t>
         </is>
       </c>
-      <c r="K10" s="4" t="inlineStr">
+      <c r="L10" s="4" t="inlineStr">
         <is>
           <t>DCAT export of the dataset (data.gov.gr/dataset/&lt;name&gt;.jsonld): theme from the EU data-theme vocabulary, format from the EU file-type vocabulary or the IANA media types, frequency from the EU frequency vocabulary.</t>
         </is>
       </c>
-      <c r="L10" s="4" t="inlineStr">
+      <c r="M10" s="4" t="inlineStr">
         <is>
           <t>all</t>
         </is>
       </c>
-      <c r="M10" s="4" t="inlineStr">
+      <c r="N10" s="4" t="inlineStr">
         <is>
           <t>Low: select the terms from the vocabularies.</t>
         </is>
       </c>
-      <c r="N10" s="4" t="inlineStr">
+      <c r="O10" s="4" t="inlineStr">
         <is>
           <t>DCAT-AP 3.0.1 (controlled vocabularies); W3C Data on the Web Best Practices (2017), BP15</t>
         </is>
       </c>
-      <c r="O10" s="4" t="inlineStr">
+      <c r="P10" s="4" t="inlineStr">
         <is>
           <t>I2</t>
+        </is>
+      </c>
+      <c r="Q10" s="4" t="inlineStr">
+        <is>
+          <t>Interoperability: format or media type from vocabulary</t>
+        </is>
+      </c>
+      <c r="R10" s="4" t="inlineStr">
+        <is>
+          <t>Distribution: format from vocabulary; media type from vocabulary</t>
         </is>
       </c>
     </row>
@@ -1253,53 +1406,68 @@
       </c>
       <c r="E11" s="3" t="inlineStr">
         <is>
+          <t>Level (b): clarity of the licence; CC BY 4.0 or a more permissive licence</t>
+        </is>
+      </c>
+      <c r="F11" s="3" t="inlineStr">
+        <is>
           <t>Is an open licence declared clearly for all resources?</t>
         </is>
       </c>
-      <c r="F11" s="3" t="inlineStr">
+      <c r="G11" s="3" t="inlineStr">
         <is>
           <t>No licence, or a licence that restricts re-use (non-commercial, no derivatives, permission required).</t>
         </is>
       </c>
-      <c r="G11" s="3" t="inlineStr">
+      <c r="H11" s="3" t="inlineStr">
         <is>
           <t>An open licence, but not declared for every resource, given only as text without a link, conflicting between resources, or more restrictive than CC BY 4.0 (e.g. share-alike).</t>
         </is>
       </c>
-      <c r="H11" s="3" t="inlineStr">
+      <c r="I11" s="3" t="inlineStr">
         <is>
           <t>Every resource carries, directly or through the dataset, the link of CC0, CC BY 4.0 or an equivalent or less restrictive open licence.</t>
         </is>
       </c>
-      <c r="I11" s="3" t="inlineStr"/>
-      <c r="J11" s="3" t="inlineStr">
+      <c r="J11" s="3" t="inlineStr"/>
+      <c r="K11" s="3" t="inlineStr">
         <is>
           <t>automatic, confirmed manually</t>
         </is>
       </c>
-      <c r="K11" s="3" t="inlineStr">
+      <c r="L11" s="3" t="inlineStr">
         <is>
           <t>Licence of the dataset and of each resource in the portal metadata; in case of conflict, the terms on the publisher's website.</t>
         </is>
       </c>
-      <c r="L11" s="3" t="inlineStr">
+      <c r="M11" s="3" t="inlineStr">
         <is>
           <t>all</t>
         </is>
       </c>
-      <c r="M11" s="3" t="inlineStr">
+      <c r="N11" s="3" t="inlineStr">
         <is>
           <t>Low: declare the licence in the metadata.</t>
         </is>
       </c>
-      <c r="N11" s="3" t="inlineStr">
+      <c r="O11" s="3" t="inlineStr">
         <is>
           <t>Directive (EU) 2019/1024, Art. 8; Regulation (EU) 2023/138, Art. 4; Ministerial Decision 11654/2026, Art. 8; W3C Data on the Web Best Practices (2017), BP4</t>
         </is>
       </c>
-      <c r="O11" s="3" t="inlineStr">
+      <c r="P11" s="3" t="inlineStr">
         <is>
           <t>R1.1</t>
+        </is>
+      </c>
+      <c r="Q11" s="3" t="inlineStr">
+        <is>
+          <t>Reusability: licence information; licence vocabulary</t>
+        </is>
+      </c>
+      <c r="R11" s="3" t="inlineStr">
+        <is>
+          <t>Distribution: license information; license vocabulary</t>
         </is>
       </c>
     </row>
@@ -1326,53 +1494,68 @@
       </c>
       <c r="E12" s="4" t="inlineStr">
         <is>
+          <t>Level (b): free of charge</t>
+        </is>
+      </c>
+      <c r="F12" s="4" t="inlineStr">
+        <is>
           <t>Can the data be obtained free of charge and without registration?</t>
         </is>
       </c>
-      <c r="F12" s="4" t="inlineStr">
+      <c r="G12" s="4" t="inlineStr">
         <is>
           <t>A charge applies, or access requires an account that is not open to everyone.</t>
         </is>
       </c>
-      <c r="G12" s="4" t="inlineStr">
+      <c r="H12" s="4" t="inlineStr">
         <is>
           <t>Free of charge, but registration, an API key or acceptance of additional terms is required.</t>
         </is>
       </c>
-      <c r="H12" s="4" t="inlineStr">
+      <c r="I12" s="4" t="inlineStr">
         <is>
           <t>Free of charge and without registration.</t>
         </is>
       </c>
-      <c r="I12" s="4" t="inlineStr"/>
-      <c r="J12" s="4" t="inlineStr">
+      <c r="J12" s="4" t="inlineStr"/>
+      <c r="K12" s="4" t="inlineStr">
         <is>
           <t>manual</t>
         </is>
       </c>
-      <c r="K12" s="4" t="inlineStr">
+      <c r="L12" s="4" t="inlineStr">
         <is>
           <t>During the download test and on the publisher's pages linked from the dataset.</t>
         </is>
       </c>
-      <c r="L12" s="4" t="inlineStr">
+      <c r="M12" s="4" t="inlineStr">
         <is>
           <t>all</t>
         </is>
       </c>
-      <c r="M12" s="4" t="inlineStr">
+      <c r="N12" s="4" t="inlineStr">
         <is>
           <t>High: change of the access policy.</t>
         </is>
       </c>
-      <c r="N12" s="4" t="inlineStr">
+      <c r="O12" s="4" t="inlineStr">
         <is>
           <t>Directive (EU) 2019/1024, Art. 6 and Art. 14; Ministerial Decision 11654/2026, Art. 8</t>
         </is>
       </c>
-      <c r="O12" s="4" t="inlineStr">
+      <c r="P12" s="4" t="inlineStr">
         <is>
           <t>A1</t>
+        </is>
+      </c>
+      <c r="Q12" s="4" t="inlineStr">
+        <is>
+          <t>Reusability: access restrictions; access restrictions vocabulary (declaration only)</t>
+        </is>
+      </c>
+      <c r="R12" s="4" t="inlineStr">
+        <is>
+          <t>Dataset: access rights; access rights vocabulary (declaration only)</t>
         </is>
       </c>
     </row>
@@ -1399,53 +1582,68 @@
       </c>
       <c r="E13" s="4" t="inlineStr">
         <is>
+          <t>Addition: Ministerial Decision 11654/2026, Art. 5</t>
+        </is>
+      </c>
+      <c r="F13" s="4" t="inlineStr">
+        <is>
           <t>How are the data made available, in the order of preference of the Ministerial Decision: API, direct link, structured file, unstructured file?</t>
         </is>
       </c>
-      <c r="F13" s="4" t="inlineStr">
+      <c r="G13" s="4" t="inlineStr">
         <is>
           <t>Only through a web page or an application without download, or no working access.</t>
         </is>
       </c>
-      <c r="G13" s="4" t="inlineStr">
+      <c r="H13" s="4" t="inlineStr">
         <is>
           <t>Files that do not give the complete data through a direct link: split into many parts, or reachable only through an intermediate page, form or map viewer.</t>
         </is>
       </c>
-      <c r="H13" s="4" t="inlineStr">
+      <c r="I13" s="4" t="inlineStr">
         <is>
           <t>An API, or a stable direct link to the complete data.</t>
         </is>
       </c>
-      <c r="I13" s="4" t="inlineStr"/>
-      <c r="J13" s="4" t="inlineStr">
+      <c r="J13" s="4" t="inlineStr"/>
+      <c r="K13" s="4" t="inlineStr">
         <is>
           <t>automatic, confirmed manually</t>
         </is>
       </c>
-      <c r="K13" s="4" t="inlineStr">
+      <c r="L13" s="4" t="inlineStr">
         <is>
           <t>Type and address of each resource (fact sheet): API or download service; direct download link; landing page or viewer.</t>
         </is>
       </c>
-      <c r="L13" s="4" t="inlineStr">
+      <c r="M13" s="4" t="inlineStr">
         <is>
           <t>all</t>
         </is>
       </c>
-      <c r="M13" s="4" t="inlineStr">
+      <c r="N13" s="4" t="inlineStr">
         <is>
           <t>Medium: publish a direct link to the complete data. High: build an API.</t>
         </is>
       </c>
-      <c r="N13" s="4" t="inlineStr">
+      <c r="O13" s="4" t="inlineStr">
         <is>
           <t>Ministerial Decision 11654/2026, Art. 5; W3C Data on the Web Best Practices (2017), BP17 and BP23</t>
         </is>
       </c>
-      <c r="O13" s="4" t="inlineStr">
+      <c r="P13" s="4" t="inlineStr">
         <is>
           <t>A1</t>
+        </is>
+      </c>
+      <c r="Q13" s="4" t="inlineStr">
+        <is>
+          <t>Accessibility: download URL (presence only)</t>
+        </is>
+      </c>
+      <c r="R13" s="4" t="inlineStr">
+        <is>
+          <t>Distribution: download URL (presence only)</t>
         </is>
       </c>
     </row>
@@ -1472,53 +1670,68 @@
       </c>
       <c r="E14" s="4" t="inlineStr">
         <is>
+          <t>Addition: FAIR F1; W3C Data on the Web Best Practices, BP9 and BP10</t>
+        </is>
+      </c>
+      <c r="F14" s="4" t="inlineStr">
+        <is>
           <t>Do the dataset and its resources have stable identifiers?</t>
         </is>
       </c>
-      <c r="F14" s="4" t="inlineStr">
+      <c r="G14" s="4" t="inlineStr">
         <is>
           <t>No stable address: the dataset or its resources are reachable only through temporary or session-based links.</t>
         </is>
       </c>
-      <c r="G14" s="4" t="inlineStr">
+      <c r="H14" s="4" t="inlineStr">
         <is>
           <t>The dataset has a stable address, but its resources point to links that change (new address with every upload, query or session parameters).</t>
         </is>
       </c>
-      <c r="H14" s="4" t="inlineStr">
+      <c r="I14" s="4" t="inlineStr">
         <is>
           <t>The dataset has a stable URI and identifier, and its resources have stable links.</t>
         </is>
       </c>
-      <c r="I14" s="4" t="inlineStr"/>
-      <c r="J14" s="4" t="inlineStr">
+      <c r="J14" s="4" t="inlineStr"/>
+      <c r="K14" s="4" t="inlineStr">
         <is>
           <t>automatic, confirmed manually</t>
         </is>
       </c>
-      <c r="K14" s="4" t="inlineStr">
+      <c r="L14" s="4" t="inlineStr">
         <is>
           <t>URI and identifier of the dataset in the DCAT export; addresses of the resources (fact sheet).</t>
         </is>
       </c>
-      <c r="L14" s="4" t="inlineStr">
+      <c r="M14" s="4" t="inlineStr">
         <is>
           <t>all</t>
         </is>
       </c>
-      <c r="M14" s="4" t="inlineStr">
+      <c r="N14" s="4" t="inlineStr">
         <is>
           <t>Low: assign stable addresses.</t>
         </is>
       </c>
-      <c r="N14" s="4" t="inlineStr">
+      <c r="O14" s="4" t="inlineStr">
         <is>
           <t>W3C Data on the Web Best Practices (2017), BP9 and BP10; DCAT-AP 3.0.1 (identifier)</t>
         </is>
       </c>
-      <c r="O14" s="4" t="inlineStr">
+      <c r="P14" s="4" t="inlineStr">
         <is>
           <t>F1</t>
+        </is>
+      </c>
+      <c r="Q14" s="4" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="R14" s="4" t="inlineStr">
+        <is>
+          <t>Dataset: identifier (dct:identifier; adms:identifier) (presence only)</t>
         </is>
       </c>
     </row>
@@ -1545,51 +1758,66 @@
       </c>
       <c r="E15" s="4" t="inlineStr">
         <is>
+          <t>Addition: legal status (GDPR; Directive (EU) 2019/1024)</t>
+        </is>
+      </c>
+      <c r="F15" s="4" t="inlineStr">
+        <is>
           <t>Does the dataset avoid exposing personal data?</t>
         </is>
       </c>
-      <c r="F15" s="4" t="inlineStr">
+      <c r="G15" s="4" t="inlineStr">
         <is>
           <t>Personal data of natural persons (names, identity or tax numbers, home addresses, personal contact details) are published without a stated legal basis.</t>
         </is>
       </c>
-      <c r="G15" s="4" t="inlineStr">
+      <c r="H15" s="4" t="inlineStr">
         <is>
           <t>Indirect identification is possible (e.g. very small counts, exact locations linked to individuals) and the dataset does not state how it was anonymised.</t>
         </is>
       </c>
-      <c r="H15" s="4" t="inlineStr">
+      <c r="I15" s="4" t="inlineStr">
         <is>
           <t>No personal data; or personal data published under a legal obligation that the metadata state; or data aggregated or anonymised, as stated.</t>
         </is>
       </c>
-      <c r="I15" s="4" t="inlineStr"/>
-      <c r="J15" s="4" t="inlineStr">
+      <c r="J15" s="4" t="inlineStr"/>
+      <c r="K15" s="4" t="inlineStr">
         <is>
           <t>manual</t>
         </is>
       </c>
-      <c r="K15" s="4" t="inlineStr">
+      <c r="L15" s="4" t="inlineStr">
         <is>
           <t>Inspection of the columns and of 10 random records; description and documentation of the dataset.</t>
         </is>
       </c>
-      <c r="L15" s="4" t="inlineStr">
+      <c r="M15" s="4" t="inlineStr">
         <is>
           <t>all</t>
         </is>
       </c>
-      <c r="M15" s="4" t="inlineStr">
+      <c r="N15" s="4" t="inlineStr">
         <is>
           <t>Medium: remove or aggregate the fields.</t>
         </is>
       </c>
-      <c r="N15" s="4" t="inlineStr">
+      <c r="O15" s="4" t="inlineStr">
         <is>
           <t>Regulation (EU) 2016/679 (GDPR); Directive (EU) 2019/1024, Art. 1(4); Ministerial Decision 11654/2026, Art. 7</t>
         </is>
       </c>
-      <c r="O15" s="4" t="inlineStr"/>
+      <c r="P15" s="4" t="inlineStr"/>
+      <c r="Q15" s="4" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="R15" s="4" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="64" customHeight="1">
       <c r="A16" s="4" t="inlineStr">
@@ -1614,61 +1842,76 @@
       </c>
       <c r="E16" s="4" t="inlineStr">
         <is>
+          <t>Addition: Regulation (EU) 2023/138, Art. 3(5)</t>
+        </is>
+      </c>
+      <c r="F16" s="4" t="inlineStr">
+        <is>
           <t>Do the metadata mark the dataset as high-value?</t>
         </is>
       </c>
-      <c r="F16" s="4" t="inlineStr">
+      <c r="G16" s="4" t="inlineStr">
         <is>
           <t>No marking: the dataset is high-value by content only.</t>
         </is>
       </c>
-      <c r="G16" s="4" t="inlineStr">
+      <c r="H16" s="4" t="inlineStr">
         <is>
           <t>Partial marking: the category without a reference to Regulation 2023/138, the reference without the category, or only the high-value dataset type.</t>
         </is>
       </c>
-      <c r="H16" s="4" t="inlineStr">
+      <c r="I16" s="4" t="inlineStr">
         <is>
           <t>High-value category and a reference to Regulation 2023/138 as applicable legislation.</t>
         </is>
       </c>
-      <c r="I16" s="4" t="inlineStr">
+      <c r="J16" s="4" t="inlineStr">
         <is>
           <t>Datasets of the comparison group.</t>
         </is>
       </c>
-      <c r="J16" s="4" t="inlineStr">
+      <c r="K16" s="4" t="inlineStr">
         <is>
           <t>automatic</t>
         </is>
       </c>
-      <c r="K16" s="4" t="inlineStr">
+      <c r="L16" s="4" t="inlineStr">
         <is>
           <t>Fields hvd_category, applicable_legislation and dcat_type of the portal metadata.</t>
         </is>
       </c>
-      <c r="L16" s="4" t="inlineStr">
+      <c r="M16" s="4" t="inlineStr">
         <is>
           <t>high-value</t>
         </is>
       </c>
-      <c r="M16" s="4" t="inlineStr">
+      <c r="N16" s="4" t="inlineStr">
         <is>
           <t>Low: complete the metadata.</t>
         </is>
       </c>
-      <c r="N16" s="4" t="inlineStr">
+      <c r="O16" s="4" t="inlineStr">
         <is>
           <t>Regulation (EU) 2023/138, Art. 3; DCAT-AP HVD</t>
         </is>
       </c>
-      <c r="O16" s="4" t="inlineStr">
+      <c r="P16" s="4" t="inlineStr">
         <is>
           <t>F2</t>
         </is>
       </c>
-    </row>
-    <row r="17" ht="49" customHeight="1">
+      <c r="Q16" s="4" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="R16" s="4" t="inlineStr">
+        <is>
+          <t>Dataset: applicable legislation (presence only)</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="139" customHeight="1">
       <c r="A17" s="4" t="inlineStr">
         <is>
           <t>M10</t>
@@ -1691,61 +1934,76 @@
       </c>
       <c r="E17" s="4" t="inlineStr">
         <is>
+          <t>Level (b): API and bulk download</t>
+        </is>
+      </c>
+      <c r="F17" s="4" t="inlineStr">
+        <is>
           <t>Is the dataset available both through an API and as a bulk download, as the Regulation requires?</t>
         </is>
       </c>
-      <c r="F17" s="4" t="inlineStr">
+      <c r="G17" s="4" t="inlineStr">
         <is>
           <t>Neither an API nor a bulk download of the complete dataset.</t>
         </is>
       </c>
-      <c r="G17" s="4" t="inlineStr">
+      <c r="H17" s="4" t="inlineStr">
         <is>
           <t>Only one of the two, or an API without public documentation and terms of use.</t>
         </is>
       </c>
-      <c r="H17" s="4" t="inlineStr">
+      <c r="I17" s="4" t="inlineStr">
         <is>
           <t>An API with public documentation and terms of use, and a bulk download of the complete dataset.</t>
         </is>
       </c>
-      <c r="I17" s="4" t="inlineStr">
+      <c r="J17" s="4" t="inlineStr">
         <is>
           <t>Datasets of the comparison group.</t>
         </is>
       </c>
-      <c r="J17" s="4" t="inlineStr">
+      <c r="K17" s="4" t="inlineStr">
         <is>
           <t>semi-automatic</t>
         </is>
       </c>
-      <c r="K17" s="4" t="inlineStr">
-        <is>
-          <t>Data services of the portal linked to the dataset (access_services), services of the publisher, and download links of the complete data.</t>
-        </is>
-      </c>
       <c r="L17" s="4" t="inlineStr">
         <is>
+          <t>Data services of the portal linked to the dataset (access_services), services of the publisher, and download links of the complete data. Exceptions of the Annex of the Regulation: numerical weather prediction (NWP) model data are required only through an API (point 3.2(a)), and historical versions of Earth observation and environment datasets through an API or a bulk download (point 2.2(a)); in these cases the required means of access alone scores 2.</t>
+        </is>
+      </c>
+      <c r="M17" s="4" t="inlineStr">
+        <is>
           <t>high-value</t>
         </is>
       </c>
-      <c r="M17" s="4" t="inlineStr">
+      <c r="N17" s="4" t="inlineStr">
         <is>
           <t>Medium: publish a complete download. High: build an API.</t>
         </is>
       </c>
-      <c r="N17" s="4" t="inlineStr">
-        <is>
-          <t>Regulation (EU) 2023/138, Art. 3 and Annex; W3C Data on the Web Best Practices (2017), BP17, BP23 and BP25</t>
-        </is>
-      </c>
       <c r="O17" s="4" t="inlineStr">
         <is>
+          <t>Regulation (EU) 2023/138, Art. 3(1) to 3(4) and Annex (exceptions in points 2.2(a) and 3.2(a)); W3C Data on the Web Best Practices (2017), BP17, BP23 and BP25</t>
+        </is>
+      </c>
+      <c r="P17" s="4" t="inlineStr">
+        <is>
           <t>A1</t>
         </is>
       </c>
-    </row>
-    <row r="18" ht="79" customHeight="1">
+      <c r="Q17" s="4" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="R17" s="4" t="inlineStr">
+        <is>
+          <t>Data service: endpoint URL; endpoint description; serves dataset. Distribution: download URL</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="109" customHeight="1">
       <c r="A18" s="5" t="inlineStr">
         <is>
           <t>AI1</t>
@@ -1768,57 +2026,72 @@
       </c>
       <c r="E18" s="6" t="inlineStr">
         <is>
+          <t>Level (c): machine readability</t>
+        </is>
+      </c>
+      <c r="F18" s="6" t="inlineStr">
+        <is>
           <t>Can a program read the data directly, without manual cleaning?</t>
         </is>
       </c>
-      <c r="F18" s="6" t="inlineStr">
+      <c r="G18" s="6" t="inlineStr">
         <is>
           <t>Not without manual work: PDF or scanned documents, images, spreadsheets laid out for printing (merged cells, several tables in one sheet), or no data file.</t>
         </is>
       </c>
-      <c r="G18" s="6" t="inlineStr">
+      <c r="H18" s="6" t="inlineStr">
         <is>
           <t>Readable after minor cleaning: title or note rows above the table, a totals row, numbers stored as text, a header split over two rows.</t>
         </is>
       </c>
-      <c r="H18" s="6" t="inlineStr">
+      <c r="I18" s="6" t="inlineStr">
         <is>
           <t>One header row, one record per row and one value per cell, without notes or totals inside the table; or a standard structured format (GeoJSON, JSON, XML) that is read without errors.</t>
         </is>
       </c>
-      <c r="I18" s="6" t="inlineStr"/>
-      <c r="J18" s="6" t="inlineStr">
+      <c r="J18" s="6" t="inlineStr"/>
+      <c r="K18" s="6" t="inlineStr">
         <is>
           <t>semi-automatic</t>
         </is>
       </c>
-      <c r="K18" s="6" t="inlineStr">
+      <c r="L18" s="6" t="inlineStr">
         <is>
           <t>Automatic read test of the most recent machine-readable file (fact sheet), then a look at the file.</t>
         </is>
       </c>
-      <c r="L18" s="6" t="inlineStr">
+      <c r="M18" s="6" t="inlineStr">
         <is>
           <t>all</t>
         </is>
       </c>
-      <c r="M18" s="6" t="inlineStr">
+      <c r="N18" s="6" t="inlineStr">
         <is>
           <t>Medium: restructure the file.</t>
         </is>
       </c>
-      <c r="N18" s="6" t="inlineStr">
-        <is>
-          <t>W3C Data on the Web Best Practices (2017), BP12; GDS (2026), Guidelines and best practices for making government datasets ready for AI; Wickham (2014), Tidy Data</t>
-        </is>
-      </c>
       <c r="O18" s="6" t="inlineStr">
         <is>
+          <t>W3C Data on the Web Best Practices (2017), BP12; GDS (2026), Guidelines and best practices for making government datasets ready for AI; Wickham (2014), Tidy Data; Publications Office of the EU (2021), data.europa.eu data quality guidelines, sections 1.2.1.2 to 1.2.1.4</t>
+        </is>
+      </c>
+      <c r="P18" s="6" t="inlineStr">
+        <is>
           <t>I1</t>
         </is>
       </c>
-    </row>
-    <row r="19" ht="94" customHeight="1">
+      <c r="Q18" s="6" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="R18" s="6" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="124" customHeight="1">
       <c r="A19" s="2" t="inlineStr">
         <is>
           <t>AI2</t>
@@ -1841,53 +2114,68 @@
       </c>
       <c r="E19" s="3" t="inlineStr">
         <is>
+          <t>Level (c): schema documentation</t>
+        </is>
+      </c>
+      <c r="F19" s="3" t="inlineStr">
+        <is>
           <t>Is the meaning, type and unit of every field documented (data dictionary)?</t>
         </is>
       </c>
-      <c r="F19" s="3" t="inlineStr">
+      <c r="G19" s="3" t="inlineStr">
         <is>
           <t>No documentation: the meaning of the fields or codes has to be guessed.</t>
         </is>
       </c>
-      <c r="G19" s="3" t="inlineStr">
+      <c r="H19" s="3" t="inlineStr">
         <is>
           <t>Partial: the field names are clear but units or codes are not explained, or only some fields are documented.</t>
         </is>
       </c>
-      <c r="H19" s="3" t="inlineStr">
+      <c r="I19" s="3" t="inlineStr">
         <is>
           <t>Every field has a description, type and unit, and the codes are explained, in the metadata, in a data dictionary or on a page linked from the metadata.</t>
         </is>
       </c>
-      <c r="I19" s="3" t="inlineStr"/>
-      <c r="J19" s="3" t="inlineStr">
+      <c r="J19" s="3" t="inlineStr"/>
+      <c r="K19" s="3" t="inlineStr">
         <is>
           <t>manual</t>
         </is>
       </c>
-      <c r="K19" s="3" t="inlineStr">
+      <c r="L19" s="3" t="inlineStr">
         <is>
           <t>Description, documentation resources and publisher pages linked from the dataset, compared with the columns of the file.</t>
         </is>
       </c>
-      <c r="L19" s="3" t="inlineStr">
+      <c r="M19" s="3" t="inlineStr">
         <is>
           <t>all</t>
         </is>
       </c>
-      <c r="M19" s="3" t="inlineStr">
+      <c r="N19" s="3" t="inlineStr">
         <is>
           <t>Low: write a data dictionary.</t>
         </is>
       </c>
-      <c r="N19" s="3" t="inlineStr">
-        <is>
-          <t>W3C Data on the Web Best Practices (2017), BP3; GDS (2026), Guidelines and best practices for making government datasets ready for AI; Gebru et al. (2021), Datasheets for Datasets; MLCommons Croissant 1.0 (RecordSet, Field)</t>
-        </is>
-      </c>
       <c r="O19" s="3" t="inlineStr">
         <is>
+          <t>W3C Data on the Web Best Practices (2017), BP3; GDS (2026), Guidelines and best practices for making government datasets ready for AI; Gebru et al. (2021), Datasheets for Datasets; MLCommons Croissant 1.0 (RecordSet, Field); Regulation (EU) 2023/138, Annex, points 2.2(c), 3.2(c), 4.2(c), 5.2(b) and 6.2(c)</t>
+        </is>
+      </c>
+      <c r="P19" s="3" t="inlineStr">
+        <is>
           <t>R1</t>
+        </is>
+      </c>
+      <c r="Q19" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="R19" s="3" t="inlineStr">
+        <is>
+          <t>Distribution: documentation (presence only)</t>
         </is>
       </c>
     </row>
@@ -1914,57 +2202,72 @@
       </c>
       <c r="E20" s="4" t="inlineStr">
         <is>
+          <t>Level (c): historical series</t>
+        </is>
+      </c>
+      <c r="F20" s="4" t="inlineStr">
+        <is>
           <t>Are earlier periods or versions of the data available?</t>
         </is>
       </c>
-      <c r="F20" s="4" t="inlineStr">
+      <c r="G20" s="4" t="inlineStr">
         <is>
           <t>Only the current state; earlier data have been replaced or removed.</t>
         </is>
       </c>
-      <c r="G20" s="4" t="inlineStr">
+      <c r="H20" s="4" t="inlineStr">
         <is>
           <t>Some earlier periods or versions, with gaps or in a different structure.</t>
         </is>
       </c>
-      <c r="H20" s="4" t="inlineStr">
+      <c r="I20" s="4" t="inlineStr">
         <is>
           <t>A continuous series of earlier periods or versions in the same structure.</t>
         </is>
       </c>
-      <c r="I20" s="4" t="inlineStr">
+      <c r="J20" s="4" t="inlineStr">
         <is>
           <t>The dataset describes a single fixed moment by design (e.g. a historical map) and is not updated.</t>
         </is>
       </c>
-      <c r="J20" s="4" t="inlineStr">
+      <c r="K20" s="4" t="inlineStr">
         <is>
           <t>manual</t>
         </is>
       </c>
-      <c r="K20" s="4" t="inlineStr">
+      <c r="L20" s="4" t="inlineStr">
         <is>
           <t>Resources per period, temporal coverage in the metadata, archive pages of the publisher.</t>
         </is>
       </c>
-      <c r="L20" s="4" t="inlineStr">
+      <c r="M20" s="4" t="inlineStr">
         <is>
           <t>all</t>
         </is>
       </c>
-      <c r="M20" s="4" t="inlineStr">
+      <c r="N20" s="4" t="inlineStr">
         <is>
           <t>Medium: publish the archive.</t>
         </is>
       </c>
-      <c r="N20" s="4" t="inlineStr">
+      <c r="O20" s="4" t="inlineStr">
         <is>
           <t>W3C Data on the Web Best Practices (2017), BP7 and BP8; GDS (2026), Guidelines and best practices for making government datasets ready for AI</t>
         </is>
       </c>
-      <c r="O20" s="4" t="inlineStr">
+      <c r="P20" s="4" t="inlineStr">
         <is>
           <t>R1</t>
+        </is>
+      </c>
+      <c r="Q20" s="4" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="R20" s="4" t="inlineStr">
+        <is>
+          <t>None</t>
         </is>
       </c>
     </row>
@@ -1991,53 +2294,68 @@
       </c>
       <c r="E21" s="4" t="inlineStr">
         <is>
+          <t>Level (c): description with Croissant or Datasheets</t>
+        </is>
+      </c>
+      <c r="F21" s="4" t="inlineStr">
+        <is>
           <t>Can the dataset be described in Croissant, or with a datasheet, from the information available?</t>
         </is>
       </c>
-      <c r="F21" s="4" t="inlineStr">
+      <c r="G21" s="4" t="inlineStr">
         <is>
           <t>Neither: a licence or a machine-readable distribution is missing, and the documentation does not say what the data contain or how they were collected.</t>
         </is>
       </c>
-      <c r="G21" s="4" t="inlineStr">
+      <c r="H21" s="4" t="inlineStr">
         <is>
           <t>A valid Croissant description at dataset level only, without the fields, or a datasheet with major gaps.</t>
         </is>
       </c>
-      <c r="H21" s="4" t="inlineStr">
+      <c r="I21" s="4" t="inlineStr">
         <is>
           <t>A valid Croissant description that includes the fields with their types and meaning, or, for data without records, a datasheet that states what the data contain, how they were collected and for which uses they are suitable.</t>
         </is>
       </c>
-      <c r="I21" s="4" t="inlineStr"/>
-      <c r="J21" s="4" t="inlineStr">
+      <c r="J21" s="4" t="inlineStr"/>
+      <c r="K21" s="4" t="inlineStr">
         <is>
           <t>semi-automatic</t>
         </is>
       </c>
-      <c r="K21" s="4" t="inlineStr">
+      <c r="L21" s="4" t="inlineStr">
         <is>
           <t>Croissant file generated from the portal metadata and the file structure and validated with the mlcroissant library; the fields are described with the information found under AI2.</t>
         </is>
       </c>
-      <c r="L21" s="4" t="inlineStr">
+      <c r="M21" s="4" t="inlineStr">
         <is>
           <t>all</t>
         </is>
       </c>
-      <c r="M21" s="4" t="inlineStr">
+      <c r="N21" s="4" t="inlineStr">
         <is>
           <t>Low: complete the metadata and the data dictionary.</t>
         </is>
       </c>
-      <c r="N21" s="4" t="inlineStr">
+      <c r="O21" s="4" t="inlineStr">
         <is>
           <t>MLCommons Croissant 1.0; Gebru et al. (2021), Datasheets for Datasets</t>
         </is>
       </c>
-      <c r="O21" s="4" t="inlineStr">
+      <c r="P21" s="4" t="inlineStr">
         <is>
           <t>R1.3</t>
+        </is>
+      </c>
+      <c r="Q21" s="4" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="R21" s="4" t="inlineStr">
+        <is>
+          <t>None</t>
         </is>
       </c>
     </row>
@@ -2064,53 +2382,68 @@
       </c>
       <c r="E22" s="4" t="inlineStr">
         <is>
+          <t>Level (c): suitability for RAG</t>
+        </is>
+      </c>
+      <c r="F22" s="4" t="inlineStr">
+        <is>
           <t>Can the content be split into self-contained pieces that an AI system can retrieve and cite?</t>
         </is>
       </c>
-      <c r="F22" s="4" t="inlineStr">
+      <c r="G22" s="4" t="inlineStr">
         <is>
           <t>Not usable: scanned images or maps without text, or no content that can be extracted.</t>
         </is>
       </c>
-      <c r="G22" s="4" t="inlineStr">
+      <c r="H22" s="4" t="inlineStr">
         <is>
           <t>Usable after conversion (text extraction from a born-digital PDF, flattening of a spreadsheet), or the pieces lack a stable identifier or a link to the source.</t>
         </is>
       </c>
-      <c r="H22" s="4" t="inlineStr">
+      <c r="I22" s="4" t="inlineStr">
         <is>
           <t>Records or text passages with a stable identifier and a link to the source, in text that is extracted cleanly in UTF-8, Greek included.</t>
         </is>
       </c>
-      <c r="I22" s="4" t="inlineStr"/>
-      <c r="J22" s="4" t="inlineStr">
+      <c r="J22" s="4" t="inlineStr"/>
+      <c r="K22" s="4" t="inlineStr">
         <is>
           <t>manual</t>
         </is>
       </c>
-      <c r="K22" s="4" t="inlineStr">
+      <c r="L22" s="4" t="inlineStr">
         <is>
           <t>Text extraction test and check of the Greek encoding (fact sheet); presence of an identifier per record.</t>
         </is>
       </c>
-      <c r="L22" s="4" t="inlineStr">
+      <c r="M22" s="4" t="inlineStr">
         <is>
           <t>all</t>
         </is>
       </c>
-      <c r="M22" s="4" t="inlineStr">
+      <c r="N22" s="4" t="inlineStr">
         <is>
           <t>Medium: publish the content as structured text or records.</t>
         </is>
       </c>
-      <c r="N22" s="4" t="inlineStr">
+      <c r="O22" s="4" t="inlineStr">
         <is>
           <t>GDS (2026), Guidelines and best practices for making government datasets ready for AI (unstructured data); W3C Data on the Web Best Practices (2017), BP10</t>
         </is>
       </c>
-      <c r="O22" s="4" t="inlineStr">
+      <c r="P22" s="4" t="inlineStr">
         <is>
           <t>F1</t>
+        </is>
+      </c>
+      <c r="Q22" s="4" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="R22" s="4" t="inlineStr">
+        <is>
+          <t>None</t>
         </is>
       </c>
     </row>
@@ -2137,53 +2470,68 @@
       </c>
       <c r="E23" s="4" t="inlineStr">
         <is>
+          <t>Addition: FAIR I3; W3C Data on the Web Best Practices, BP10 and BP15</t>
+        </is>
+      </c>
+      <c r="F23" s="4" t="inlineStr">
+        <is>
           <t>Can the data be joined with other datasets through common codes or coordinates?</t>
         </is>
       </c>
-      <c r="F23" s="4" t="inlineStr">
+      <c r="G23" s="4" t="inlineStr">
         <is>
           <t>No identifiers or location information that allow linkage.</t>
         </is>
       </c>
-      <c r="G23" s="4" t="inlineStr">
+      <c r="H23" s="4" t="inlineStr">
         <is>
           <t>Only names (e.g. municipality names) or codes internal to the publisher, or coordinates without a declared reference system.</t>
         </is>
       </c>
-      <c r="H23" s="4" t="inlineStr">
+      <c r="I23" s="4" t="inlineStr">
         <is>
           <t>Standard codes (e.g. municipality codes of the Kallikratis classification, NUTS or LAU codes, KAD/NACE activity codes, tax or GEMI numbers, KAEK cadastral codes) or coordinates in a declared reference system.</t>
         </is>
       </c>
-      <c r="I23" s="4" t="inlineStr"/>
-      <c r="J23" s="4" t="inlineStr">
+      <c r="J23" s="4" t="inlineStr"/>
+      <c r="K23" s="4" t="inlineStr">
         <is>
           <t>semi-automatic</t>
         </is>
       </c>
-      <c r="K23" s="4" t="inlineStr">
+      <c r="L23" s="4" t="inlineStr">
         <is>
           <t>Column names and values (fact sheet); reference system of the geospatial files.</t>
         </is>
       </c>
-      <c r="L23" s="4" t="inlineStr">
+      <c r="M23" s="4" t="inlineStr">
         <is>
           <t>all</t>
         </is>
       </c>
-      <c r="M23" s="4" t="inlineStr">
+      <c r="N23" s="4" t="inlineStr">
         <is>
           <t>Medium: add the standard codes.</t>
         </is>
       </c>
-      <c r="N23" s="4" t="inlineStr">
+      <c r="O23" s="4" t="inlineStr">
         <is>
           <t>W3C Data on the Web Best Practices (2017), BP10 and BP15; FAIR I3</t>
         </is>
       </c>
-      <c r="O23" s="4" t="inlineStr">
+      <c r="P23" s="4" t="inlineStr">
         <is>
           <t>I3</t>
+        </is>
+      </c>
+      <c r="Q23" s="4" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="R23" s="4" t="inlineStr">
+        <is>
+          <t>None</t>
         </is>
       </c>
     </row>
@@ -2210,58 +2558,73 @@
       </c>
       <c r="E24" s="4" t="inlineStr">
         <is>
+          <t>Addition: Datasheets for Datasets; GDS (2026)</t>
+        </is>
+      </c>
+      <c r="F24" s="4" t="inlineStr">
+        <is>
           <t>Do the metadata or the documentation state the known limitations of the data?</t>
         </is>
       </c>
-      <c r="F24" s="4" t="inlineStr">
+      <c r="G24" s="4" t="inlineStr">
         <is>
           <t>No statement about coverage, gaps, collection method or known errors.</t>
         </is>
       </c>
-      <c r="G24" s="4" t="inlineStr">
+      <c r="H24" s="4" t="inlineStr">
         <is>
           <t>A partial statement, e.g. only the source or only the coverage.</t>
         </is>
       </c>
-      <c r="H24" s="4" t="inlineStr">
+      <c r="I24" s="4" t="inlineStr">
         <is>
           <t>Coverage, gaps, collection method and known errors or changes of method are stated.</t>
         </is>
       </c>
-      <c r="I24" s="4" t="inlineStr"/>
-      <c r="J24" s="4" t="inlineStr">
+      <c r="J24" s="4" t="inlineStr"/>
+      <c r="K24" s="4" t="inlineStr">
         <is>
           <t>manual</t>
         </is>
       </c>
-      <c r="K24" s="4" t="inlineStr">
+      <c r="L24" s="4" t="inlineStr">
         <is>
           <t>Description, documentation resources and linked publisher pages.</t>
         </is>
       </c>
-      <c r="L24" s="4" t="inlineStr">
+      <c r="M24" s="4" t="inlineStr">
         <is>
           <t>all</t>
         </is>
       </c>
-      <c r="M24" s="4" t="inlineStr">
+      <c r="N24" s="4" t="inlineStr">
         <is>
           <t>Low: add a short note on limitations.</t>
         </is>
       </c>
-      <c r="N24" s="4" t="inlineStr">
+      <c r="O24" s="4" t="inlineStr">
         <is>
           <t>Gebru et al. (2021), Datasheets for Datasets; GDS (2026), Guidelines and best practices for making government datasets ready for AI; W3C Data on the Web Best Practices (2017), BP6</t>
         </is>
       </c>
-      <c r="O24" s="4" t="inlineStr">
+      <c r="P24" s="4" t="inlineStr">
         <is>
           <t>R1.2</t>
         </is>
       </c>
+      <c r="Q24" s="4" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="R24" s="4" t="inlineStr">
+        <is>
+          <t>Dataset: provenance (presence only)</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:O24"/>
+  <autoFilter ref="A1:R24"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
 </worksheet>
@@ -2273,7 +2636,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A7"/>
+  <dimension ref="A1:A9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="110" customWidth="1" min="1" max="1"/>
@@ -2313,12 +2676,26 @@
     <row r="6" ht="34" customHeight="1">
       <c r="A6" s="8" t="inlineStr">
         <is>
+          <t>Instruction: the point of the written instructions of the supervisor that the criterion implements. 'Addition' marks a criterion added to those points, followed by its source.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="49" customHeight="1">
+      <c r="A7" s="8" t="inlineStr">
+        <is>
+          <t>MQA: the indicators of the Metadata Quality Assessment that check the same aspect as the criterion, in the previous methodology, applied by data.gov.gr, and in the current methodology of data.europa.eu. 'None' marks a criterion that no indicator covers.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="34" customHeight="1">
+      <c r="A8" s="8" t="inlineStr">
+        <is>
           <t>Effort of a fix: low (metadata and documentation only), medium (a change in the file itself), high (a change in a system or in the source of the data).</t>
         </is>
       </c>
     </row>
-    <row r="7" ht="19" customHeight="1">
-      <c r="A7" s="8" t="inlineStr">
+    <row r="9" ht="19" customHeight="1">
+      <c r="A9" s="8" t="inlineStr">
         <is>
           <t>Full rules: criteria/README.md.</t>
         </is>

</xml_diff>